<commit_message>
Cleanup temporary batch 6 completion scripts
</commit_message>
<xml_diff>
--- a/data/extracted_100_brand_new_100k_500k_batch7.xlsx
+++ b/data/extracted_100_brand_new_100k_500k_batch7.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q68"/>
+  <dimension ref="A1:Q70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5808,6 +5808,164 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>mandanazarghami</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Mandana Zarghami</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>mandanazarghami1@gmail.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>136K</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>135700</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Celebrity &amp; Public Figure</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Miami, FL, US</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Miami Lifestyle Creator</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mandanazarghami</t>
+        </is>
+      </c>
+      <c r="K69" t="b">
+        <v>1</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>$1,500</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>1 Instagram Photo Feed Post</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>https://hoo.be/mandanazarghami</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:16:21Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>kwin</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Cat</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>kwinandre@gmail.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>104K</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>103600</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Music &amp; Dance</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Miami, FL, US</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Entertainment, artist, lifestyle</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kwin</t>
+        </is>
+      </c>
+      <c r="K70" t="b">
+        <v>1</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>1 Instagram Story</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>https://taplink.cc/kwin</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:16:28Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Synchronize batch dataset files
</commit_message>
<xml_diff>
--- a/data/extracted_100_brand_new_100k_500k_batch7.xlsx
+++ b/data/extracted_100_brand_new_100k_500k_batch7.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q70"/>
+  <dimension ref="A1:Q72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5966,6 +5966,164 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>welcometothepeasantparty</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Charlotte Warren</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>welcometothepeasantparty@gmail.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>251K</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>250700</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Austin, TX, US</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Dating &amp; Relationships Content Creator</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/welcometothepeasantparty</t>
+        </is>
+      </c>
+      <c r="K71" t="b">
+        <v>1</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>$300</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>1 TikTok Video (60 Seconds)</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>https://hoo.be/welcometothepeasantparty</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:17:33Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>kirabarbie</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Kira Barbie</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>kiralovestravel@gmail.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>119K</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>118900</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>New York, NY, US</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Travel Content Creator</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kirabarbie</t>
+        </is>
+      </c>
+      <c r="K72" t="b">
+        <v>1</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>$1,000</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>1 TikTok Video (30 Seconds)</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>https://msha.ke/kirabarbie</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:18:20Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update batch 6 excel dataset
</commit_message>
<xml_diff>
--- a/data/extracted_100_brand_new_100k_500k_batch7.xlsx
+++ b/data/extracted_100_brand_new_100k_500k_batch7.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q72"/>
+  <dimension ref="A1:Q73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6124,6 +6124,85 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>gera</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Geraldine Linares</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>anatolijzinkovskij05@gmail.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>102K</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>101600</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Boston, MA, US</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Entertainer and health advocate</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/gera</t>
+        </is>
+      </c>
+      <c r="K73" t="b">
+        <v>1</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>$300</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>https://taplink.cc/gera</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>2026-09-18T13:20:28Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete 100 Batch 7 creators & push to Supabase DB (Live count: 1310)
</commit_message>
<xml_diff>
--- a/data/extracted_100_brand_new_100k_500k_batch7.xlsx
+++ b/data/extracted_100_brand_new_100k_500k_batch7.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q73"/>
+  <dimension ref="A1:Q91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6203,6 +6203,1428 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>godsayz</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>God's Messages</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>godsayzbusiness@gmail.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>459K</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>458700</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>New York, NY, US</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Faith-Based &amp; Motivational Content Creator | High Engagement | US Audience</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/godsayz</t>
+        </is>
+      </c>
+      <c r="K74" t="b">
+        <v>1</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>$50</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>1 Instagram Story</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/godsayz</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>2026-09-18T14:32:22Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>andrewphysics</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Andrew Gomez</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>andrewphysics@mail.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>227K</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>227000</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>El Paso, TX, US</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Artist, Streamer, Online Weirdo</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/andrewphysics</t>
+        </is>
+      </c>
+      <c r="K75" t="b">
+        <v>1</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>$299</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/andrewphysics</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:48:12Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>whitcharae</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Whitney Creamer</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>whitcharae@outlook.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>365K</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>365200</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Del Rio, TX, US</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Beauty content creator</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/whitcharae</t>
+        </is>
+      </c>
+      <c r="K76" t="b">
+        <v>1</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>$350</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>1 TikTok Video (60 Seconds)</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>https://beacons.ai/whitcharae</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:48:13Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>vicmram</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Victor Ramos</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>victor@vicmram.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>231K</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>230800</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>LGBTQ2+</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, US</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Entertainment and Lifestyle Content Creator</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/vicmram</t>
+        </is>
+      </c>
+      <c r="K77" t="b">
+        <v>1</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>1 Instagram Story</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/vicmram</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:48:27Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>apopofyou</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Katelyn Collier</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>apopofyoudesigns@gmail.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>233K</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>232800</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Home &amp; Garden</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Chesapeake, VA, US</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Parenting and Education Content Creator</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/apopofyou</t>
+        </is>
+      </c>
+      <c r="K78" t="b">
+        <v>1</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/apopofyou</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:48:28Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>parissenpai</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Paris Senpai</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>paristhesenpai@gmail.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>308K</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>308200</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Orlando, FL, US</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Content Creator, Model, Influencer</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/parissenpai</t>
+        </is>
+      </c>
+      <c r="K79" t="b">
+        <v>1</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>$450</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>1 Instagram Story</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/parissenpai</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:48:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>timonsdreams</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Xcm</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>xcmbus@gmail.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>185K</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>185300</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Comedy &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, US</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Anime comedy creator specializing in storytelling and animation</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/timonsdreams</t>
+        </is>
+      </c>
+      <c r="K80" t="b">
+        <v>1</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>1 Instagram Story</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/timonsdreams</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:51:18Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>annaknows</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Ganna Ignatenko</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>annaknows30@gmail.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>140K</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>139700</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Home &amp; Garden</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Moore, SC, US</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Home Improvement and Lifestyle Tips Expert</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/annaknows</t>
+        </is>
+      </c>
+      <c r="K81" t="b">
+        <v>1</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>$70</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>1 TikTok Story</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/annaknows</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:56:35Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>pineapplehoneydew</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Pineapple Honeydew</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>madison@pineapplehoneydew.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>133K</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>133000</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA, US</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>🏳️‍⚧️ It Girl and Funny Lady</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/pineapplehoneydew</t>
+        </is>
+      </c>
+      <c r="K82" t="b">
+        <v>1</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>$150</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>1 TikTok Story</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/pineapplehoneydew</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:58:36Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>chefstuart</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Stuart Okeeffe</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>chefstuartla@gmail.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>300K</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>299900</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Celebrity &amp; Public Figure</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, US</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Chef Stuart O'Keeffe – Celebrity chef and content creator</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/chefstuart</t>
+        </is>
+      </c>
+      <c r="K83" t="b">
+        <v>1</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>1 Instagram Story</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/chefstuart</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>2026-09-19T06:59:19Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>lifewithmichelle</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Michelle Henderson</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>hello@lifewithmichelle.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>122K</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>122500</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Outdoor &amp; Nature</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, US</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Lifestyle Content Creator</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lifewithmichelle</t>
+        </is>
+      </c>
+      <c r="K84" t="b">
+        <v>1</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>$240</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>1 Instagram Photo Feed Post</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>https://stan.store/lifewithmichelle</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:00:09Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>leahvanderpool</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Leah Vanderpool</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>leahbieber930015@gmail.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>201K</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>200900</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Cleveland, OH, US</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Lifestyle &amp; Travel Creator</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/leahvanderpool</t>
+        </is>
+      </c>
+      <c r="K85" t="b">
+        <v>1</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>$100</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>1 TikTok Story</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>https://hoo.be/leahvanderpool</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:00:10Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ethemedium</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ethemedium@gmail.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>233K</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>233300</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>DIY &amp; Craft</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>New York, NY, US</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Intuitive Psychic Live Streamer Sharing Spiritual Insights</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/ethemedium</t>
+        </is>
+      </c>
+      <c r="K86" t="b">
+        <v>1</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>$750</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>1 TikTok Video</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/ethemedium</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:00:52Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>nursecharles</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Nurse Charles</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>partnerships@nursecharlesmedia.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>128K</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>128199</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>DIY &amp; Craft</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>ER Nurse and Health Coach</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nursecharles</t>
+        </is>
+      </c>
+      <c r="K87" t="b">
+        <v>1</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>1 TikTok Story</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/nursecharles</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:00:53Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>landofmma</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Charlie Bergin</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>landofmma@gmail.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>175K</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>175300</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Athlete &amp; Sports</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Harrisville, RI, US</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>MMA content creator</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/landofmma</t>
+        </is>
+      </c>
+      <c r="K88" t="b">
+        <v>1</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>$50</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/landofmma</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:01:37Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>amberforbes</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Amber Forbes</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>amberforbespr@gmail.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>150K</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>150100</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Relatable Travel and Lifestyle Influencer</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/amberforbes</t>
+        </is>
+      </c>
+      <c r="K89" t="b">
+        <v>1</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>$500</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>1 TikTok Video (15 Seconds)</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>https://stan.store/amberforbes</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:06:16Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>theemoodyfoody</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Fabrizio Villalpando</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>emma.lux@thedigitalbrandarchitects.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>240K</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>240300</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Home &amp; Garden</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, US</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Fine dining waiter turned home cook - 6%+ IG engagement. TikTok verified.</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/theemoodyfoody</t>
+        </is>
+      </c>
+      <c r="K90" t="b">
+        <v>1</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>$2,000</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>1 Instagram Photo Feed Post</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>https://beacons.ai/theemoodyfoody</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:12:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>gerardiperformance</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Michaelangelo Gerardi</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>mike@gerardiperformance.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>149K</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>149200</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Entrepreneur &amp; Business</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Boston, MA, US</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Fitness Content Creator and Personal Trainer</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/gerardiperformance</t>
+        </is>
+      </c>
+      <c r="K91" t="b">
+        <v>1</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>$150</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>1 Instagram Story</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>https://hoo.be/gerardiperformance</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:17:39Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Finalize Batch 7 dataset (100 creators, 100k-500k USA)
</commit_message>
<xml_diff>
--- a/data/extracted_100_brand_new_100k_500k_batch7.xlsx
+++ b/data/extracted_100_brand_new_100k_500k_batch7.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q91"/>
+  <dimension ref="A1:Q101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -523,7 +523,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Promote with Itsbrendas</t>
+          <t>Itsbrendas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -602,7 +602,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Promote with Gabriela Paz</t>
+          <t>Gabriela Paz</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Promote with Eric Guilmette</t>
+          <t>Eric Guilmette</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Promote with Gabby Mata</t>
+          <t>Gabby Mata</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Promote with Douie</t>
+          <t>Douie</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Promote with Cindy Maureen</t>
+          <t>Cindy Maureen</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -997,7 +997,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Promote with Max</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Promote with Kat V</t>
+          <t>Kat V</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Promote with Cass And Alexa Meade</t>
+          <t>Cass And Alexa Meade</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Promote with Kayley Burnett</t>
+          <t>Kayley Burnett</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Promote with Kylee Mroz</t>
+          <t>Kylee Mroz</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Promote with Adrian Johnson</t>
+          <t>Adrian Johnson</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Promote with Cassie Lee</t>
+          <t>Cassie Lee</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -7622,6 +7622,796 @@
       <c r="Q91" t="inlineStr">
         <is>
           <t>2026-09-19T07:17:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>cutieefoodie</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Megan Sri</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>milktea.meg1@gmail.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>132K</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>132300</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Food &amp; Drink</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Los Angeles, CA, US</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Passionate about beauty and fashion!</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/cutieefoodie</t>
+        </is>
+      </c>
+      <c r="K92" t="b">
+        <v>1</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>$1,200</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>https://beacons.ai/cutieefoodie</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:20:29.498538+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>nailsbydianamichelle</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Nailsbydianamichelle</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>michelledianapr@gmail.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>104K</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>104100</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Art &amp; Photography</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Carteret, NJ, US</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Nail Artist &amp; Content Creator</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nailsbydianamichelle</t>
+        </is>
+      </c>
+      <c r="K93" t="b">
+        <v>1</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>$300</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>1 TikTok Video (60 Seconds)</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>https://stan.store/nailsbydianamichelle</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:23:49.143336+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>krystalaranyani</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Krystal Aranyani</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>love@krystal-aranyani.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>102K</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>101900</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Comedy &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Sacramento, CA, US</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Author, Feminine Empowerment, Spirituality &amp; Wellness Coach</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/krystalaranyani</t>
+        </is>
+      </c>
+      <c r="K94" t="b">
+        <v>1</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>$250</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>https://hoo.be/krystalaranyani</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:29:36.072182+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>natalialevsina</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Natalia Levsina</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>hello@allbuenothings.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>186K</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>185900</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Travel</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>New York, NY, US</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>NYC-based influencer, who covers such topics as fashion, beauty, travel,etc</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/natalialevsina</t>
+        </is>
+      </c>
+      <c r="K95" t="b">
+        <v>1</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>$1,000</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>https://beacons.ai/natalialevsina</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:31:16.297834+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>thedriversclub</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Matthew Forde</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>webmail@thedriversclub.de</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>481K</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>481400</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Tampa, FL, US</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Automotive</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/thedriversclub</t>
+        </is>
+      </c>
+      <c r="K96" t="b">
+        <v>1</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>$2,000</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/thedriversclub</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:32:54.779322+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>floridaguidejosh</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Josh Swander</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>joshuamswander@gmail.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>102K</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>101800</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Ocala, FL, US</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Wildlife Educator, Photographer, &amp; Content Creator</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/floridaguidejosh</t>
+        </is>
+      </c>
+      <c r="K97" t="b">
+        <v>1</v>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>$450</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>1 TikTok Video</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/floridaguidejosh</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:34:35.308146+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>chanceperez</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>chanceperezbusiness@gmail.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>282K</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>281800</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Music &amp; Dance</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Los Alamitos, CA, US</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Lifestyle, Family and Fitness</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/chanceperez</t>
+        </is>
+      </c>
+      <c r="K98" t="b">
+        <v>1</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>$1,200</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>1 TikTok Story</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/chanceperez</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:35:24.805328+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>noeahjacobs</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Noeah Jacobs</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>noeahtrinity@gmail.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>126K</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>125700</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Comedy &amp; Entertainment</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Palm Beach, FL, US</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Streetwear model, dancer, content creator</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/noeahjacobs</t>
+        </is>
+      </c>
+      <c r="K99" t="b">
+        <v>1</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>$800</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>1 Instagram Photo Feed Post</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>https://hoo.be/noeahjacobs</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:36:18.037976+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>victorianpoetry</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Victorian Poetry</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>victorianerastories@aol.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>412K</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>412300</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Music &amp; Dance</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Rochester, NY, US</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Poetry Content Creator</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/victorianpoetry</t>
+        </is>
+      </c>
+      <c r="K100" t="b">
+        <v>1</v>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>$400</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>1 TikTok Video</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/victorianpoetry</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:39:28.76352+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>lateologiadelacalle</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Carlos M Irizarry</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>info@lateologiadelacalle.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>159K</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>159000</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>DIY &amp; Craft</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Miami, FL, US</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Urban &amp; Christian Content Creator + Farruko's Content Creator</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lateologiadelacalle</t>
+        </is>
+      </c>
+      <c r="K101" t="b">
+        <v>1</v>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>$1,188</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>1 Instagram Reel</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>https://linktr.ee/lateologiadelacalle</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>not_sent</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>2026-09-19T07:40:17.227992+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>